<commit_message>
Format log workbook as bordered tables
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/logs/trading_logs.xlsx
+++ b/logs/trading_logs.xlsx
@@ -56,7 +56,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -68,8 +68,13 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF2F8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -77,13 +82,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9D6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C9D6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C9D6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,8 +473,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -467,7 +495,7 @@
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,248 +581,248 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
@@ -803,14 +831,16 @@
   </sheetData>
   <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -827,7 +857,7 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
@@ -839,7 +869,7 @@
     <col width="32" customWidth="1" min="22" max="22"/>
     <col width="34" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="60" customWidth="1" min="25" max="25"/>
+    <col width="55" customWidth="1" min="25" max="25"/>
     <col width="28" customWidth="1" min="26" max="26"/>
     <col width="19" customWidth="1" min="27" max="27"/>
   </cols>
@@ -982,275 +1012,275 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>8c5b446c-b9e6-5f4d-9dd8-1599063963d8</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>NEEDS_REVIEW</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Legacy record retained; not automatically regraded because its timestamps and candle-boundary semantics are not verified.</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>market_predictions_log.csv</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>99f129c6-c768-5c75-b98d-b263bb633309</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>NEEDS_REVIEW</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
+      <c r="T3" s="3" t="inlineStr"/>
+      <c r="U3" s="3" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
+      <c r="W3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr"/>
+      <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>Legacy record retained; not automatically regraded because its timestamps and candle-boundary semantics are not verified.</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z3" s="3" t="inlineStr">
         <is>
           <t>market_predictions_log.csv</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA3" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>e195c1a6-6c1b-5503-926e-11d1f36b2872</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:58:40+00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>81260.86</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:30:00+00:00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T13:58:40+00:00</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>81650.0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>81150.0</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>81520.0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Following a healthy pullback to test the rising 15-minute moving average support near 81,200, buyers are stepping back in with RSI resetting to a balanced 58.7. Over the next two hours, price is expected to resume its prevailing macro uptrend and retest the recent swing high area between 81,500 and 81,650.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>NEEDS_REVIEW</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>Legacy record retained; not automatically regraded because its timestamps and candle-boundary semantics are not verified.</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>market_predictions_log.csv</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1259,14 +1289,16 @@
   </sheetData>
   <autoFilter ref="A1:AA4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1283,7 +1315,7 @@
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
@@ -1378,221 +1410,221 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:58:40+00:00</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:58:40+00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:30:00+00:00</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T13:58:40+00:00</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>81260.86</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>81150.0</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>81650.0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>81520.0</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Following a healthy pullback to test the rising 15-minute moving average support near 81,200, buyers are stepping back in with RSI resetting to a balanced 58.7. Over the next two hours, price is expected to resume its prevailing macro uptrend and retest the recent swing high area between 81,500 and 81,650.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -1601,14 +1633,16 @@
   </sheetData>
   <autoFilter ref="A1:Q4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1686,14 +1720,16 @@
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1706,9 +1742,9 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1769,290 +1805,290 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
@@ -2061,14 +2097,16 @@
   </sheetData>
   <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2088,7 +2126,7 @@
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2174,248 +2212,248 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
@@ -2424,20 +2462,22 @@
   </sheetData>
   <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2453,680 +2493,680 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>[2026-10-28T01:18:37] Gatekeeper triggered.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>[DATA] Fetching BTC-USD spot candles (4h, 15d)...</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">python.exe : D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:568: Pandas4Warning: The inplace keyword in </t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>DataFrame.sort_index is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>At line:2 char:1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>+ &amp; '.\venv\Scripts\python.exe' -u '.\auto_run.py' *&gt; '.\auto_run.log'</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>+ ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">    + CategoryInfo          : NotSpecified: (D:\trading agen...rsion (PDEP-8).:String) [], RemoteException</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    + FullyQualifiedErrorId : NativeCommandError</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  quotes.sort_index(inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:514: Pandas4Warning: The inplace keyword in DataFrame.drop </t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  df.drop(</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:518: Pandas4Warning: The inplace keyword in DataFrame.rename </t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  df.rename(columns={</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\multi.py:220: Pandas4Warning: The inplace keyword in DataFrame.rename </t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  data.rename(columns=ctx.isins, inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\multi.py:224: Pandas4Warning: The inplace keyword in </t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>DataFrame.sort_index is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  data.sort_index(level=0, axis=1, inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>[DATA] Retrieved 88 spot candles.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>[DATA] Compiling market context...</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>[DATA] Fetching US Dollar Index (DX-Y.NYB)...</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:568: Pandas4Warning: The inplace keyword in </t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>DataFrame.sort_index is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  quotes.sort_index(inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:514: Pandas4Warning: The inplace keyword in DataFrame.drop </t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  df.drop(</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\utils.py:518: Pandas4Warning: The inplace keyword in DataFrame.rename </t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>43</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  df.rename(columns={</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\multi.py:220: Pandas4Warning: The inplace keyword in DataFrame.rename </t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>48</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  data.rename(columns=ctx.isins, inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D:\trading agent\venv\Lib\site-packages\yfinance\multi.py:224: Pandas4Warning: The inplace keyword in </t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>DataFrame.sort_index is deprecated and will be removed in a future version (PDEP-8).</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>51</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>See https://pandas.pydata.org/docs/dev/whatsnew/v3.1.0.html#deprecation-inplace for more details.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  data.sort_index(level=0, axis=1, inplace=True)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>[DATA] DXY close=102.2840, daily change=0.3178%.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>[DATA] Fetching Binance futures data for BTCUSDT...</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>[DATA] Open interest=96603.815, annualized funding=10.9500%.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>[DATA] Market context compiled.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>findfont: Failed to find font weight semibold for DejaVu Sans, now using 700.</t>
         </is>
@@ -3135,14 +3175,16 @@
   </sheetData>
   <autoFilter ref="A1:B58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3162,7 +3204,7 @@
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3248,248 +3290,248 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
@@ -3498,14 +3540,16 @@
   </sheetData>
   <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3525,7 +3569,7 @@
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3611,248 +3655,248 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
@@ -3861,14 +3905,16 @@
   </sheetData>
   <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3885,7 +3931,7 @@
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
@@ -3980,221 +4026,221 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:58:40+00:00</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:58:40+00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T11:30:00+00:00</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-10-28T13:58:40+00:00</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>81260.86</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>81150.0</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>81650.0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>81520.0</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Following a healthy pullback to test the rising 15-minute moving average support near 81,200, buyers are stepping back in with RSI resetting to a balanced 58.7. Over the next two hours, price is expected to resume its prevailing macro uptrend and retest the recent swing high area between 81,500 and 81,650.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -4203,14 +4249,16 @@
   </sheetData>
   <autoFilter ref="A1:Q4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4223,9 +4271,9 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4286,290 +4334,290 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
@@ -4578,14 +4626,16 @@
   </sheetData>
   <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4598,9 +4648,9 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4661,290 +4711,290 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
@@ -4953,14 +5003,16 @@
   </sheetData>
   <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4973,9 +5025,9 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5036,290 +5088,290 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 02:20:25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>81399.99</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>81120.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>81550.0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Price is currently experiencing a low-volume relief bounce into the declining 15m EMAs between 81,420 and 81,520. As the macro trend remains bearish and RSI sits below 50, overhead dynamic resistance is expected to reject this advance. Over the next 2 hours, price will likely stall near resistance and rotate back downward to retest the recent swing low around 81,145.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-24 18:01:24</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>80680.29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>The current 15-minute bounce is testing dynamic moving average resistance near the recent swing high of 80800. Due to strong prevailing bearish momentum on the 1-hour macro chart, this relief rally is likely to stall and face rejection. Expect price to fade back toward local support near 80450-80500 over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24 18:04:36</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>80656.49</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>80420.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>80820.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>BTC-USD is rebounding from local support near 80,350 but faces immediate dynamic resistance from the declining short-term moving averages near 80,700-80,800. Due to prevailing macro bearish momentum coupled with a cooling bounce, price is likely to be capped below the 80,816 swing high. Expect a chop-heavy consolidation within the 80,420 to 80,820 range over the next 2 hours.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-25 01:27:51</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>80397.58</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>79850.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>80600.0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Legacy</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not graded</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Following an aggressive V-shaped recovery into overhead resistance near 80,500-80,600, the 15-minute RSI is severely overbought at 82.35 within an established 1-hour macro downtrend. Upward momentum is stalling with upper wicks forming below prior support-turned-resistance. Expect price to face rejection and retrace lower toward the 80,000 psychological level and underlying short-term moving average over the next two hours.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-10-26 16:26:54</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>80328.69</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>80180.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>80680.0</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>80520.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Following a strong impulse above the 80,000 level, the price is consolidating tightly in a bullish flag pattern above the 15-minute moving average. Over the next 2 hours, price is expected to hold above the 80,200 support and break out past the 80,462 swing high to challenge the 80,650 resistance zone.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 00:44:00</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>79865.69</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>79450.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>80150.0</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>79620.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Price is breaking down below the key psychological level of 80000 following a lower high rejection on both 1H and 15m timeframes. With the 15m RSI at 33.42 confirming downward momentum, any brief pullbacks toward 80050 are likely to be sold off. Expect BTC-USD to drift lower over the next 2 hours to test liquidity near the 79450–79600 support zone.</t>
         </is>
@@ -5328,5 +5380,6 @@
   </sheetData>
   <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>